<commit_message>
Update output data files after bug fix
</commit_message>
<xml_diff>
--- a/data/imdb_data.xlsx
+++ b/data/imdb_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mehmetborataskin/Desktop/2025_03_31_imdb_project_final/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0608E07A-29AE-1147-A1FC-D776FF51533A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBFEF810-18C2-2B4F-8D29-77324F3E44FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Popular Movies" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="175">
   <si>
     <t>Popularity</t>
   </si>
@@ -114,7 +114,7 @@
     <t>Predator: Badlands</t>
   </si>
   <si>
-    <t>Set on the Predator home-world, Predator: Badlands features a complete written and verbal Predator language created by Paul R. Frommer, the linguist who developed the Na'vi language for Avatar (2009). Dimitrius Schuster-Koloamatangi, who plays the lead Predator, Dek, learned the language for the role and delivered his lines while wearing a full Predator suit created by Alec Gillis. However, unlike previous Predator films, Dek's face is CGI rather than animatronic to allowing the actor's facial performance to be conveyed via motion capture.</t>
+    <t>Set on the Predator home-world, Predator: Badlands features a complete written and verbal Predator language created by Paul R. Frommer, the linguist who developed the Na'vi language for Avatar (2009). Dimitrius Schuster-Koloamatangi, who plays the lead Predator, Dek, learned the language for the role and delivered his lines while wearing a full Predator suit created by Alec Gillis. However, unlike previous Predator films, Dek's face is CGI rather than animatronic, allowing the actor's facial performance to be conveyed via motion capture.</t>
   </si>
   <si>
     <t>This is not a sequel to the 2022 movie Prey, but it is set within the Predator universe.</t>
@@ -144,7 +144,7 @@
     <t>Steven Yeun was originally cast as Robert Reynolds/Sentry, but after filming was delayed due to the SAG-AFTRA strikes (2023), Yeun dropped out due to scheduling conflicts and was later replaced with Lewis Pullman. He later expressed disappointment of not being able to do the film, and hopes to be cast in another Marvel movie.</t>
   </si>
   <si>
-    <t>Will conclude Phase 5 of the Marvel Cinematic Universe.</t>
+    <t>According to director Jake Schreier, he used blast shadows (a phenomenon where a nuclear blast can eradicate people but leave behind their shadows burned into the ground/wall) as part of the Void's shadow powers for their simplicity and horror.</t>
   </si>
   <si>
     <t>Until Dawn</t>
@@ -237,7 +237,7 @@
     <t>Locked</t>
   </si>
   <si>
-    <t>Thriller, Bill Skarsgård, Anthony Hopkins</t>
+    <t>Thriller</t>
   </si>
   <si>
     <t>Bill Skarsgård, Anthony Hopkins, Ashley Cartwright, Michael Eklund</t>
@@ -255,7 +255,7 @@
     <t>June and John</t>
   </si>
   <si>
-    <t>Romance, Thriller, Matilda Price</t>
+    <t>Romance, Thriller</t>
   </si>
   <si>
     <t>Matilda Price, Luke Stanton Eddy, Ryan Shoos, Dean Testerman</t>
@@ -273,7 +273,7 @@
     <t>Hysteria</t>
   </si>
   <si>
-    <t>Drama, Thriller, Devrim Lingnau</t>
+    <t>Drama, Thriller</t>
   </si>
   <si>
     <t>Devrim Lingnau, Mehdi Meskar, Serkan Kaya, Nicolette Krebitz</t>
@@ -282,7 +282,7 @@
     <t>Ölü Mevsim</t>
   </si>
   <si>
-    <t>Drama, Funda Eryigit, Ece Yasar</t>
+    <t>Drama</t>
   </si>
   <si>
     <t>Funda Eryigit, Ece Yasar, Erdem Senocak, Serkan Ercan</t>
@@ -291,7 +291,7 @@
     <t>The Glory of Life</t>
   </si>
   <si>
-    <t>Drama, Romance, Henriette Confurius</t>
+    <t>Drama, Romance</t>
   </si>
   <si>
     <t>Henriette Confurius, Sabin Tambrea, Manuel Rubey, Daniela Golpashin</t>
@@ -300,7 +300,7 @@
     <t>Köstebekgiller: Ata Tohumu Muhafizlari</t>
   </si>
   <si>
-    <t>Family, Beren Gökyildiz, Pelin Akil</t>
+    <t>Family</t>
   </si>
   <si>
     <t>Beren Gökyildiz, Pelin Akil, Mehmet Aybars Kaya, Jennifer Boyner</t>
@@ -309,7 +309,7 @@
     <t>Asagi Mahalle</t>
   </si>
   <si>
-    <t>Comedy, Soner Türker, Abidin Yerebakan</t>
+    <t>Comedy</t>
   </si>
   <si>
     <t>Soner Türker, Abidin Yerebakan, Caner Atacan, Izzet Çivril</t>
@@ -318,7 +318,7 @@
     <t>Cahim</t>
   </si>
   <si>
-    <t>Horror, A. Murat Özgen, Asli Bankoglu</t>
+    <t>Horror</t>
   </si>
   <si>
     <t>A. Murat Özgen, Asli Bankoglu, Miray Arikan Aydin, Seda Sönmez</t>
@@ -330,9 +330,6 @@
     <t>Popeye the Slayer Man</t>
   </si>
   <si>
-    <t>Horror, Jason Robert Stephens, Angela Relucio</t>
-  </si>
-  <si>
     <t>Jason Robert Stephens, Angela Relucio, Sarah Nicklin, Elena Juliano</t>
   </si>
   <si>
@@ -366,25 +363,19 @@
     <t>Son Durak: Kan Bağı</t>
   </si>
   <si>
-    <t>Horror, Tony Todd, Brec Bassinger</t>
-  </si>
-  <si>
     <t>Tony Todd, Brec Bassinger, April Telek, Richard Harmon</t>
   </si>
   <si>
     <t>Hurry Up Tomorrow</t>
   </si>
   <si>
-    <t>Thriller, The Weeknd, Jenna Ortega</t>
-  </si>
-  <si>
     <t>The Weeknd, Jenna Ortega, Barry Keoghan, Riley Keough</t>
   </si>
   <si>
     <t>Riff Raff</t>
   </si>
   <si>
-    <t>Comedy, Crime, Jennifer Coolidge</t>
+    <t>Comedy, Crime</t>
   </si>
   <si>
     <t>Jennifer Coolidge, Ed Harris, Gabrielle Union, Miles J. Harvey</t>
@@ -402,9 +393,6 @@
     <t>Gülizar</t>
   </si>
   <si>
-    <t>Drama, Bekir Behrem, Asli Içözü</t>
-  </si>
-  <si>
     <t>Bekir Behrem, Asli Içözü, Ernest Malazogu, Ecem Uzun</t>
   </si>
   <si>
@@ -417,15 +405,36 @@
     <t>Full Article Link</t>
   </si>
   <si>
+    <t>Adam Pearson Will Play Joseph Merrick in New Adaptation of ‘The Elehpant Man’ from A24</t>
+  </si>
+  <si>
+    <t>In 1977, Bernard Pomerance wrote the play The Elephant Man, which became a massive hit. The play about the life of Joseph Merrick, a severely disfigured man whose life is still a fascinating mystery, became a massive hit and showed us just how we, as a society, can fail when it comes to those who are the most vulnerable.</t>
+  </si>
+  <si>
+    <t>5/1/2025</t>
+  </si>
+  <si>
+    <t>https://www.comicbasics.com/adam-pearson-will-play-joseph-merrick-in-new-adaptation-of-the-elehpant-man-from-a24/</t>
+  </si>
+  <si>
+    <t>Chris Hemsworth to Star in Amazon MGM Deep Sea Thriller ‘Subversion’</t>
+  </si>
+  <si>
+    <t>Chris Hemsworth is set to star in the Amazon MGM deep sea thriller “Subversion,” which will be produced by Lorenzo di Bonaventura.</t>
+  </si>
+  <si>
+    <t>4/30/2025</t>
+  </si>
+  <si>
+    <t>https://www.thewrap.com/chris-hemsworth-amazon-mgm-subversion/</t>
+  </si>
+  <si>
     <t>Guy Ritchie to Direct ‘Road House 2’ With Jake Gyllenhaal</t>
   </si>
   <si>
     <t>Guy Ritchie will direct the sequel to “Road House” with Jake Gyllenhaal set to reprise his lead role as ex-UFC fighter Dalton.</t>
   </si>
   <si>
-    <t>4/30/2025</t>
-  </si>
-  <si>
     <t>https://variety.com/2025/film/news/road-house-2-guy-ritchie-direct-jake-gyllenhaal-1236360265/</t>
   </si>
   <si>
@@ -450,115 +459,94 @@
     <t>https://www.thewrap.com/cbs-ratings-most-watched-network-primetime-viewers/</t>
   </si>
   <si>
-    <t>Natasha Lyonne’s Feature Directorial Debut Will Be a ‘Hybrid’ AI Movie</t>
-  </si>
-  <si>
-    <t>Natasha Lyonne is set to make her feature directorial debut — with a big assist from artificial intelligence.</t>
-  </si>
-  <si>
-    <t>https://www.thewrap.com/natasha-lyonne-directorial-debut-ai-movie/</t>
-  </si>
-  <si>
-    <t>‘A Minecraft Movie’ Stays on Top as ‘Sinners’ Holds Strong and ‘Star Wars: Revenge of the Sith’ Reissue Blasts Into Third at U.K. and Ireland Box Office</t>
-  </si>
-  <si>
-    <t>Warner Bros.’ “A Minecraft Movie” continues its domination at the U.K. and Ireland box office, topping the chart for a fourth straight weekend with £2.4 million ($3.3 million), according to Comscore. The film has amassed $68.7 million to date, firmly establishing itself as one of the biggest hits of 2025.</t>
-  </si>
-  <si>
-    <t>https://variety.com/2025/film/box-office/a-minecraft-movie-uk-ireland-box-office-4-1236381035/</t>
-  </si>
-  <si>
-    <t>Tony Awards Nominations: Denzel Washington and Jake Gyllenhaal’s ‘Othello’ Shut Out Despite Strong Ticket Sales</t>
-  </si>
-  <si>
-    <t>Othello, starring Jake Gyllenhaal and Denzel Washington, was entirely shut out of the 2025 Tony Award nominations.</t>
-  </si>
-  <si>
-    <t>5/1/2025</t>
-  </si>
-  <si>
-    <t>https://www.hollywoodreporter.com/lifestyle/arts/2025-tony-awards-nominations-snubs-surprises-1236204998/</t>
-  </si>
-  <si>
-    <t>Ari Emanuel to Buy Frieze as Endeavor Sell-Off Continues</t>
-  </si>
-  <si>
-    <t>With the Silver Lake take-private complete, Endeavor Group Holdings continues to sell off its remaining “non-core” assets, with Ari Emanuel still the biggest buyer.</t>
-  </si>
-  <si>
-    <t>https://www.hollywoodreporter.com/business/business-news/ari-emanuel-buys-frieze-art-fair-endeavor-sell-off-1236204994/</t>
-  </si>
-  <si>
-    <t>2025 Tony Awards: ‘Buena Vista Social Club,’ ‘Death Becomes Her,’ ‘Maybe Happy Ending’ Lead Nominations</t>
-  </si>
-  <si>
-    <t>Musicals Buena Vista Social Club, Death Becomes Her and Maybe Happy Ending lead the 2025 Tony nominations with 10 nods each.</t>
-  </si>
-  <si>
-    <t>https://www.hollywoodreporter.com/lifestyle/arts/2025-tony-awards-nominees-full-list-nominations-1236204935/</t>
-  </si>
-  <si>
-    <t>2025 Tony Nominations: ‘Buena Vista Social Club,’ ‘Death Becomes Her’ and ‘Maybe Happy Ending’ Lead With 10 Nods Each</t>
-  </si>
-  <si>
-    <t>In one of the most crowded, celebrity-propelled Broadway seasons in recent memory, three musicals — two based upon popular movies — emerged supreme amongst Tony nominators in 2025, banking an impressive 10 nods each.</t>
-  </si>
-  <si>
-    <t>https://www.thewrap.com/tony-nominations-2025-complete-list/</t>
-  </si>
-  <si>
-    <t>100 Days of Trump: MSNBC and CNN Trudge to Pre-Election Numbers as Fox News Grows</t>
-  </si>
-  <si>
-    <t>While the aftermath of Donald Trump’s win in the 2024 election saw some grim ratings for MSNBC and CNN, viewership for the cable news networks is slowly trudging back to pre-election numbers, while Fox News’ audience continues to grow 100 days into his second term.</t>
-  </si>
-  <si>
-    <t>https://www.thewrap.com/100-days-trump-cable-news-ratings-msnbc-cnn-fox-news/</t>
-  </si>
-  <si>
-    <t>Family-Vlogger Documentary Trend Magnifies a Serious Societal Problem</t>
-  </si>
-  <si>
-    <t>Recent documentaries like Hulu’s Devil in the Family: The Fall of Ruby Franke and Netflix’s Bad Influence: The Dark Side of Kidfluencing should have society — or at least social media — shook. Both projects shine a spotlight on abuses of minors in the hugely popular family-vlogging space. Behind the shiny-happy presentation of children, tweens and teens is a mostly-unregulated environment that can bend (if not completely breaks) child labor laws, enable online predators and create unknown damage to the psyche of developing brains.</t>
-  </si>
-  <si>
-    <t>https://www.hollywoodreporter.com/business/digital/family-vlogger-documentary-trend-serious-societal-problem-1236198669/</t>
-  </si>
-  <si>
-    <t>How to Watch the 2025 Tony Awards Nominations Live</t>
-  </si>
-  <si>
-    <t>The 2025 Tony nominations are here.</t>
-  </si>
-  <si>
-    <t>https://www.hollywoodreporter.com/lifestyle/arts/how-to-watch-2025-tony-awards-nominations-live-1236204371/</t>
-  </si>
-  <si>
-    <t>New Nyt Games Feature Will Let Fans Play Wordle Against Celebs Laufey, Lola Tung, Chris Perfetti, Luann de Lesseps and Sonja Morgan (Exclusive)</t>
-  </si>
-  <si>
-    <t>The New York Times Games app debuted a new leaderboard feature last month that allows users to check their performance against friends. Now, the makers of Wordle, Connections, Spelling Bee and the Mini Crossword are giving players a chance to compare their scores with some of Nyt Games’ “most dedicated celebrity puzzlers.”</t>
-  </si>
-  <si>
-    <t>https://variety.com/2025/tv/news/nyt-games-leaderboard-celebs-laufey-lola-tung-1236382990/</t>
-  </si>
-  <si>
-    <t>Done+Dusted Expands in Middle East, Opens Saudi Office Led by Clare Baarda (Exclusive)</t>
-  </si>
-  <si>
-    <t>Pantheon Media Group’s production shingle Done+Dusted has launched an office in Saudi Arabia, appointing veteran executive Clare Baarda to serve as country manager. Baarda, whose hire was announced Thursday, will report to Done+Dusted Group CEO Simon Pizey, and reps the latest expansion for the company in the Middle East.</t>
-  </si>
-  <si>
-    <t>https://variety.com/2025/tv/news/done-dusted-saudi-office-led-by-clare-baarda-1236383018/</t>
-  </si>
-  <si>
-    <t>Can Netflix Reach the $1 Trillion Club by 2030?</t>
-  </si>
-  <si>
-    <t>With Netflix looking beyond the streaming wars and its stock price hitting new all-time highs, the company’s executives have set their sights on a new long-term target: reach a market capitalization of $1 trillion by 2030.</t>
-  </si>
-  <si>
-    <t>https://www.thewrap.com/can-netflix-reach-1-trillion-market-cap-2030-analysis/</t>
+    <t>Sarah Michelle Gellar Says Chloé Zhao’s Passion for ‘Buffy’ Changed Her Mind About a Reboot: ‘Ok, There’s a Reason’</t>
+  </si>
+  <si>
+    <t>Sarah Michelle Gellar is detailing how Academy Award winner Chloé Zhao changed her mind about a “Buffy the Vampire Slayer” reboot.</t>
+  </si>
+  <si>
+    <t>https://www.indiewire.com/news/general-news/sarah-michelle-gellar-chloe-zhao-changed-mind-buffy-reboot-1235119630/</t>
+  </si>
+  <si>
+    <t>Willem Dafoe to Star in Dark Comedy ‘The Souffleur’ From Rising Helmer Gastón Solnicki; Magnify Boards for Worldwide Sales (Exclusive)</t>
+  </si>
+  <si>
+    <t>Willem Dafoe has signed on to star in “The Souffleur,” an English-language dark comedy directed by rising Argentinian director Gastón Solnicki. Magnify has boarded worldwide sales (excluding Austria) ahead of the Cannes Film Market. Variety has been given exclusive access to a first-look image for the film (below), which is currently in post-production.</t>
+  </si>
+  <si>
+    <t>https://variety.com/2025/film/global/willem-dafoe-the-souffleur-magnify-1236383477/</t>
+  </si>
+  <si>
+    <t>DC’s ‘Sgt. Rock’ Movie, From Luca Guadagnino, No Longer in Development</t>
+  </si>
+  <si>
+    <t>DC Studios’ “Sgt. Rock” is going on leave — but it may not be permanent.</t>
+  </si>
+  <si>
+    <t>https://variety.com/2025/film/news/sgt-rock-luca-guadagnino-dc-studios-not-in-development-1236382859/</t>
+  </si>
+  <si>
+    <t>Box Office: Chris Hemsworth, Halle Berry’s ‘Crime 101′ Lands Presidents’ Day Weekend 2026 Release (Exclusive)</t>
+  </si>
+  <si>
+    <t>Chris Hemsworth and Halle Berry‘s heist movie Crime 101 has landed a high-profile release date in theaters.</t>
+  </si>
+  <si>
+    <t>https://www.hollywoodreporter.com/movies/movie-news/chris-hemsworth-halle-berry-crime-101-2026-release-1236204739/</t>
+  </si>
+  <si>
+    <t>Takashi Miike starts filming Bad Lieutenant: Tokyo this month</t>
+  </si>
+  <si>
+    <t>Takashi Miike, the Japanese director behind films such as Audition and Ichi the Killer, has lined up his next picture, Bad Lieutenant: Tokyo, which will offer an international twist on the series that first caused controversy back in 1992 via Abel Ferrara and Harvey Keitel.</t>
+  </si>
+  <si>
+    <t>https://www.joblo.com/takashi-miike-bad-lieutenant-tokyo/</t>
+  </si>
+  <si>
+    <t>Lily James to Lead Thriller ‘Photo Booth’ for ‘Walk the Line,’ ‘Girl Interrupted’ Producer Cathy Konrad</t>
+  </si>
+  <si>
+    <t>Lily James is set to star in and produce “Photo Booth,” the directorial feature debut of Australian sibling filmmakers Spencer and Lloyd Harvey.</t>
+  </si>
+  <si>
+    <t>https://variety.com/2025/film/global/lily-james-emotional-thriller-photo-booth-1236383531/</t>
+  </si>
+  <si>
+    <t>‘The View’ Lands First Post-White House Interview With Joe and Jill Biden</t>
+  </si>
+  <si>
+    <t>Former President Joe Biden and first lady Dr. Jill Biden will sit for their first TV interview since leaving the White House on The View.</t>
+  </si>
+  <si>
+    <t>https://www.hollywoodreporter.com/tv/tv-news/joe-jill-biden-the-view-interview-1236205157/</t>
+  </si>
+  <si>
+    <t>Ariana Grande, Cynthia Erivo, Chappell Roan to Guest Judge ‘RuPaul’s Drag Race All Stars 10’</t>
+  </si>
+  <si>
+    <t>The cast of “RuPaul’s Drag Race All Stars” Season 10 was already stacked — but the new list of guest judges is downright star-studded.</t>
+  </si>
+  <si>
+    <t>https://www.thewrap.com/rupauls-drag-race-all-stars-10-guest-judges-ariana-grande-cynthia-erivo/</t>
+  </si>
+  <si>
+    <t>Embattled ’60 Minutes’ Kamala Harris Interview Among Nominees for 2025 News and Doc Emmys</t>
+  </si>
+  <si>
+    <t>CBS’ long-running “60 Minutes” has been nominated for 13 News &amp; Documentary Emmy Awards, which the National Academy of Television Arts &amp; Sciences announced on Thursday.</t>
+  </si>
+  <si>
+    <t>https://www.thewrap.com/60-minutes-kamala-harris-news-and-documentary-emmys-nominees/</t>
+  </si>
+  <si>
+    <t>Ad-Supported Platforms Account for 72.4% of TV Viewing in First Quarter of 2025</t>
+  </si>
+  <si>
+    <t>Nielsen has expanded its TV viewership measurement reports for broadcast, cable and streaming with the launch of the Ad-Supported Gauge.</t>
+  </si>
+  <si>
+    <t>https://www.thewrap.com/nielsen-ad-supported-gauge-q1-2025/</t>
   </si>
 </sst>
 </file>
@@ -577,6 +565,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1209,6 +1198,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="58.1640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
@@ -1366,108 +1361,108 @@
         <v>101</v>
       </c>
       <c r="C13" t="s">
+        <v>98</v>
+      </c>
+      <c r="D13" t="s">
         <v>102</v>
-      </c>
-      <c r="D13" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" s="3"/>
       <c r="B14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C14" t="s">
         <v>74</v>
       </c>
       <c r="D14" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="3"/>
       <c r="B15" t="s">
+        <v>105</v>
+      </c>
+      <c r="C15" t="s">
         <v>106</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>107</v>
-      </c>
-      <c r="D15" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="3"/>
       <c r="B16" t="s">
+        <v>108</v>
+      </c>
+      <c r="C16" t="s">
         <v>109</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>110</v>
-      </c>
-      <c r="D16" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B17" t="s">
         <v>112</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
+        <v>98</v>
+      </c>
+      <c r="D17" t="s">
         <v>113</v>
-      </c>
-      <c r="C17" t="s">
-        <v>114</v>
-      </c>
-      <c r="D17" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="3"/>
       <c r="B18" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C18" t="s">
-        <v>117</v>
+        <v>71</v>
       </c>
       <c r="D18" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="3"/>
       <c r="B19" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C19" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D19" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="3"/>
       <c r="B20" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C20" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="D20" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="3"/>
       <c r="B21" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C21" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
       <c r="D21" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -1484,25 +1479,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="2" max="2" width="116" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>64</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>63</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -1510,16 +1502,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C2" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="D2" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="E2" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -1527,16 +1519,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C3" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D3" t="s">
         <v>133</v>
       </c>
       <c r="E3" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -1544,16 +1536,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C4" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D4" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="E4" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -1561,16 +1553,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C5" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E5" t="s">
         <v>140</v>
-      </c>
-      <c r="E5" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -1578,16 +1570,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C6" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="D6" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="E6" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -1595,16 +1587,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C7" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D7" t="s">
-        <v>150</v>
+        <v>129</v>
       </c>
       <c r="E7" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -1612,16 +1604,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="C8" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="D8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E8" t="s">
         <v>150</v>
-      </c>
-      <c r="E8" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -1629,16 +1621,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C9" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="D9" t="s">
-        <v>150</v>
+        <v>133</v>
       </c>
       <c r="E9" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
@@ -1646,16 +1638,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="C10" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="D10" t="s">
-        <v>150</v>
+        <v>129</v>
       </c>
       <c r="E10" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
@@ -1663,16 +1655,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C11" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="D11" t="s">
-        <v>150</v>
+        <v>129</v>
       </c>
       <c r="E11" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
@@ -1680,16 +1672,16 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C12" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="D12" t="s">
-        <v>150</v>
+        <v>129</v>
       </c>
       <c r="E12" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
@@ -1697,16 +1689,16 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C13" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D13" t="s">
-        <v>150</v>
+        <v>129</v>
       </c>
       <c r="E13" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
@@ -1714,16 +1706,16 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C14" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="D14" t="s">
-        <v>150</v>
+        <v>129</v>
       </c>
       <c r="E14" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
@@ -1731,16 +1723,16 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C15" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="D15" t="s">
-        <v>150</v>
+        <v>129</v>
       </c>
       <c r="E15" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
@@ -1748,16 +1740,16 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="C16" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D16" t="s">
-        <v>150</v>
+        <v>129</v>
       </c>
       <c r="E16" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>

</xml_diff>